<commit_message>
Valor de referência passa a ser a mediana das cotações
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016bmexAMEyfJuuzawG4ELwH
</commit_message>
<xml_diff>
--- a/Cotacao_Servicos_Saude_Unidade_Movel_2026-10-07.xlsx
+++ b/Cotacao_Servicos_Saude_Unidade_Movel_2026-10-07.xlsx
@@ -61,7 +61,7 @@
     <t xml:space="preserve">VALOR GLOBAL ESTIMADO</t>
   </si>
   <si>
-    <t xml:space="preserve">Metodologia: para cada item foram reunidos três preços de contratações públicas (credenciamentos, pregões, atas de registro de preços, contratos e tabelas de credenciamento de órgãos e consórcios públicos), indicados nas colunas Fonte/Valor/Link de cada lote, com menor, média, mediana e maior valor. O valor unitário de referência de cada item é o valor adotado pela Administração para o credenciamento, aplicado uniformemente a todos os credenciados, e foi confrontado com as cotações para verificar sua compatibilidade com o mercado. Itens marcados como 'análogo' usam procedimento equivalente quando não havia o item idêntico na fonte. Os quantitativos são estimativas do TR e não geram obrigação de execução.</t>
+    <t xml:space="preserve">Metodologia: para cada item foram reunidos até três preços de contratações públicas (credenciamentos, pregões, atas de registro de preços, contratos e tabelas de credenciamento de órgãos e consórcios públicos), indicados nas colunas Fonte/Valor/Link de cada lote. O valor unitário de referência de cada item corresponde à MEDIANA dos preços coletados (Lei nº 14.133/2021, art. 23; IN SEGES/ME nº 65/2021, art. 6º), apresentada ao lado do menor preço, da média e do maior preço. Itens marcados como 'análogo' usam procedimento equivalente quando não havia o item idêntico na fonte. Itens com menos de três preços estão sujeitos à justificativa prevista no art. 6º, §5º, da IN SEGES/ME nº 65/2021. Os quantitativos são estimativas do TR e não geram obrigação de execução.</t>
   </si>
   <si>
     <t xml:space="preserve">LOTE 1 – EXAMES DE MAMOGRAFIA BILATERAL (unidade móvel)</t>
@@ -118,7 +118,7 @@
     <t xml:space="preserve">Maior (R$)</t>
   </si>
   <si>
-    <t xml:space="preserve">Valor unit. referência (R$)</t>
+    <t xml:space="preserve">Valor unit. referência (R$) = mediana</t>
   </si>
   <si>
     <t xml:space="preserve">Valor total estimado (R$)</t>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">'Lote 1 - Mamografia'!S4</f>
-        <v>4665118</v>
+        <v>4615986</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">'Lote 2 - Consultas'!S18</f>
-        <v>22774370.25</v>
+        <v>22868454.05</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">'Lote 3 - Exames'!S12</f>
-        <v>18905067.11</v>
+        <v>20674426.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">'Lote 4 - Ressonancia'!S5</f>
-        <v>11650694.4</v>
+        <v>11851030</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">'Lote 5 - Odontologia'!S67</f>
-        <v>24700500.24</v>
+        <v>20579182.67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">SUM(B6:B10)</f>
-        <v>82695750</v>
+        <v>80589079.52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1538,11 +1538,12 @@
         <v>140.45</v>
       </c>
       <c r="R3" s="14" t="n">
-        <v>134.83</v>
+        <f aca="false">IF(COUNT(F3,I3,L3)=0,"Sem cotação",ROUND(P3,2))</f>
+        <v>133.41</v>
       </c>
       <c r="S3" s="12" t="n">
-        <f aca="false">D3*R3</f>
-        <v>4665118</v>
+        <f aca="false">IF(ISNUMBER(R3),D3*R3,0)</f>
+        <v>4615986</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,7 +1569,7 @@
       <c r="R4" s="15"/>
       <c r="S4" s="7" t="n">
         <f aca="false">SUM(S3:S3)</f>
-        <v>4665118</v>
+        <v>4615986</v>
       </c>
     </row>
   </sheetData>
@@ -1755,11 +1756,12 @@
         <v>100</v>
       </c>
       <c r="R3" s="14" t="n">
-        <v>93</v>
+        <f aca="false">IF(COUNT(F3,I3,L3)=0,"Sem cotação",ROUND(P3,2))</f>
+        <v>92.48</v>
       </c>
       <c r="S3" s="12" t="n">
-        <f aca="false">D3*R3</f>
-        <v>4039920</v>
+        <f aca="false">IF(ISNUMBER(R3),D3*R3,0)</f>
+        <v>4017331.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1819,11 +1821,12 @@
         <v>115</v>
       </c>
       <c r="R4" s="14" t="n">
-        <v>95.31</v>
+        <f aca="false">IF(COUNT(F4,I4,L4)=0,"Sem cotação",ROUND(P4,2))</f>
+        <v>97.63</v>
       </c>
       <c r="S4" s="12" t="n">
-        <f aca="false">D4*R4</f>
-        <v>2846433.15</v>
+        <f aca="false">IF(ISNUMBER(R4),D4*R4,0)</f>
+        <v>2915719.95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1883,11 +1886,12 @@
         <v>125.24</v>
       </c>
       <c r="R5" s="14" t="n">
-        <v>97.62</v>
+        <f aca="false">IF(COUNT(F5,I5,L5)=0,"Sem cotação",ROUND(P5,2))</f>
+        <v>100</v>
       </c>
       <c r="S5" s="12" t="n">
-        <f aca="false">D5*R5</f>
-        <v>2385344.7</v>
+        <f aca="false">IF(ISNUMBER(R5),D5*R5,0)</f>
+        <v>2443500</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1947,11 +1951,12 @@
         <v>115</v>
       </c>
       <c r="R6" s="14" t="n">
-        <v>107.59</v>
+        <f aca="false">IF(COUNT(F6,I6,L6)=0,"Sem cotação",ROUND(P6,2))</f>
+        <v>114.97</v>
       </c>
       <c r="S6" s="12" t="n">
-        <f aca="false">D6*R6</f>
-        <v>2336854.8</v>
+        <f aca="false">IF(ISNUMBER(R6),D6*R6,0)</f>
+        <v>2497148.4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2011,11 +2016,12 @@
         <v>161.67</v>
       </c>
       <c r="R7" s="14" t="n">
-        <v>92.64</v>
+        <f aca="false">IF(COUNT(F7,I7,L7)=0,"Sem cotação",ROUND(P7,2))</f>
+        <v>96.5</v>
       </c>
       <c r="S7" s="12" t="n">
-        <f aca="false">D7*R7</f>
-        <v>2012140.8</v>
+        <f aca="false">IF(ISNUMBER(R7),D7*R7,0)</f>
+        <v>2095980</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2075,11 +2081,12 @@
         <v>115</v>
       </c>
       <c r="R8" s="14" t="n">
-        <v>95.31</v>
+        <f aca="false">IF(COUNT(F8,I8,L8)=0,"Sem cotação",ROUND(P8,2))</f>
+        <v>103.2</v>
       </c>
       <c r="S8" s="12" t="n">
-        <f aca="false">D8*R8</f>
-        <v>1380088.8</v>
+        <f aca="false">IF(ISNUMBER(R8),D8*R8,0)</f>
+        <v>1494336</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2139,11 +2146,12 @@
         <v>115</v>
       </c>
       <c r="R9" s="14" t="n">
-        <v>112.64</v>
+        <f aca="false">IF(COUNT(F9,I9,L9)=0,"Sem cotação",ROUND(P9,2))</f>
+        <v>101.56</v>
       </c>
       <c r="S9" s="12" t="n">
-        <f aca="false">D9*R9</f>
-        <v>1529088</v>
+        <f aca="false">IF(ISNUMBER(R9),D9*R9,0)</f>
+        <v>1378677</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,11 +2211,12 @@
         <v>116.67</v>
       </c>
       <c r="R10" s="14" t="n">
-        <v>112.64</v>
+        <f aca="false">IF(COUNT(F10,I10,L10)=0,"Sem cotação",ROUND(P10,2))</f>
+        <v>115</v>
       </c>
       <c r="S10" s="12" t="n">
-        <f aca="false">D10*R10</f>
-        <v>1427148.8</v>
+        <f aca="false">IF(ISNUMBER(R10),D10*R10,0)</f>
+        <v>1457050</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2267,11 +2276,12 @@
         <v>115</v>
       </c>
       <c r="R11" s="14" t="n">
-        <v>112.64</v>
+        <f aca="false">IF(COUNT(F11,I11,L11)=0,"Sem cotação",ROUND(P11,2))</f>
+        <v>90</v>
       </c>
       <c r="S11" s="12" t="n">
-        <f aca="false">D11*R11</f>
-        <v>1325209.6</v>
+        <f aca="false">IF(ISNUMBER(R11),D11*R11,0)</f>
+        <v>1058850</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2331,11 +2341,12 @@
         <v>115</v>
       </c>
       <c r="R12" s="14" t="n">
-        <v>112.64</v>
+        <f aca="false">IF(COUNT(F12,I12,L12)=0,"Sem cotação",ROUND(P12,2))</f>
+        <v>105.87</v>
       </c>
       <c r="S12" s="12" t="n">
-        <f aca="false">D12*R12</f>
-        <v>1223270.4</v>
+        <f aca="false">IF(ISNUMBER(R12),D12*R12,0)</f>
+        <v>1149748.2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2395,11 +2406,12 @@
         <v>115</v>
       </c>
       <c r="R13" s="14" t="n">
-        <v>93</v>
+        <f aca="false">IF(COUNT(F13,I13,L13)=0,"Sem cotação",ROUND(P13,2))</f>
+        <v>106.1</v>
       </c>
       <c r="S13" s="12" t="n">
-        <f aca="false">D13*R13</f>
-        <v>925815</v>
+        <f aca="false">IF(ISNUMBER(R13),D13*R13,0)</f>
+        <v>1056225.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2459,11 +2471,12 @@
         <v>115</v>
       </c>
       <c r="R14" s="14" t="n">
-        <v>93.72</v>
+        <f aca="false">IF(COUNT(F14,I14,L14)=0,"Sem cotação",ROUND(P14,2))</f>
+        <v>97.63</v>
       </c>
       <c r="S14" s="12" t="n">
-        <f aca="false">D14*R14</f>
-        <v>339266.4</v>
+        <f aca="false">IF(ISNUMBER(R14),D14*R14,0)</f>
+        <v>353420.6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2523,11 +2536,12 @@
         <v>115</v>
       </c>
       <c r="R15" s="14" t="n">
-        <v>104.7</v>
+        <f aca="false">IF(COUNT(F15,I15,L15)=0,"Sem cotação",ROUND(P15,2))</f>
+        <v>90</v>
       </c>
       <c r="S15" s="12" t="n">
-        <f aca="false">D15*R15</f>
-        <v>284260.5</v>
+        <f aca="false">IF(ISNUMBER(R15),D15*R15,0)</f>
+        <v>244350</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2587,11 +2601,12 @@
         <v>115</v>
       </c>
       <c r="R16" s="14" t="n">
-        <v>95.31</v>
+        <f aca="false">IF(COUNT(F16,I16,L16)=0,"Sem cotação",ROUND(P16,2))</f>
+        <v>91.96</v>
       </c>
       <c r="S16" s="12" t="n">
-        <f aca="false">D16*R16</f>
-        <v>517533.3</v>
+        <f aca="false">IF(ISNUMBER(R16),D16*R16,0)</f>
+        <v>499342.8</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2651,11 +2666,12 @@
         <v>161.67</v>
       </c>
       <c r="R17" s="14" t="n">
-        <v>93</v>
+        <f aca="false">IF(COUNT(F17,I17,L17)=0,"Sem cotação",ROUND(P17,2))</f>
+        <v>95.2</v>
       </c>
       <c r="S17" s="12" t="n">
-        <f aca="false">D17*R17</f>
-        <v>201996</v>
+        <f aca="false">IF(ISNUMBER(R17),D17*R17,0)</f>
+        <v>206774.4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2681,7 +2697,7 @@
       <c r="R18" s="15"/>
       <c r="S18" s="7" t="n">
         <f aca="false">SUM(S3:S17)</f>
-        <v>22774370.25</v>
+        <v>22868454.05</v>
       </c>
     </row>
   </sheetData>
@@ -2910,11 +2926,12 @@
         <v>136.91</v>
       </c>
       <c r="R3" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F3,I3,L3)=0,"Sem cotação",ROUND(P3,2))</f>
+        <v>115.05</v>
       </c>
       <c r="S3" s="12" t="n">
-        <f aca="false">D3*R3</f>
-        <v>5536640</v>
+        <f aca="false">IF(ISNUMBER(R3),D3*R3,0)</f>
+        <v>7547280</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2974,11 +2991,12 @@
         <v>150</v>
       </c>
       <c r="R4" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F4,I4,L4)=0,"Sem cotação",ROUND(P4,2))</f>
+        <v>90</v>
       </c>
       <c r="S4" s="12" t="n">
-        <f aca="false">D4*R4</f>
-        <v>882824</v>
+        <f aca="false">IF(ISNUMBER(R4),D4*R4,0)</f>
+        <v>941400</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3038,11 +3056,12 @@
         <v>135</v>
       </c>
       <c r="R5" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F5,I5,L5)=0,"Sem cotação",ROUND(P5,2))</f>
+        <v>89.72</v>
       </c>
       <c r="S5" s="12" t="n">
-        <f aca="false">D5*R5</f>
-        <v>1799830</v>
+        <f aca="false">IF(ISNUMBER(R5),D5*R5,0)</f>
+        <v>1913279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,11 +3121,12 @@
         <v>90</v>
       </c>
       <c r="R6" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F6,I6,L6)=0,"Sem cotação",ROUND(P6,2))</f>
+        <v>85.72</v>
       </c>
       <c r="S6" s="12" t="n">
-        <f aca="false">D6*R6</f>
-        <v>882824</v>
+        <f aca="false">IF(ISNUMBER(R6),D6*R6,0)</f>
+        <v>896631.2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3166,11 +3186,12 @@
         <v>244.92</v>
       </c>
       <c r="R7" s="14" t="n">
-        <v>273.31</v>
+        <f aca="false">IF(COUNT(F7,I7,L7)=0,"Sem cotação",ROUND(P7,2))</f>
+        <v>211.26</v>
       </c>
       <c r="S7" s="12" t="n">
-        <f aca="false">D7*R7</f>
-        <v>4068219.35</v>
+        <f aca="false">IF(ISNUMBER(R7),D7*R7,0)</f>
+        <v>3144605.1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3230,11 +3251,12 @@
         <v>187.17</v>
       </c>
       <c r="R8" s="14" t="n">
-        <v>122.24</v>
+        <f aca="false">IF(COUNT(F8,I8,L8)=0,"Sem cotação",ROUND(P8,2))</f>
+        <v>75</v>
       </c>
       <c r="S8" s="12" t="n">
-        <f aca="false">D8*R8</f>
-        <v>387989.76</v>
+        <f aca="false">IF(ISNUMBER(R8),D8*R8,0)</f>
+        <v>238050</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3294,11 +3316,12 @@
         <v>90.74</v>
       </c>
       <c r="R9" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F9,I9,L9)=0,"Sem cotação",ROUND(P9,2))</f>
+        <v>90</v>
       </c>
       <c r="S9" s="12" t="n">
-        <f aca="false">D9*R9</f>
-        <v>381910</v>
+        <f aca="false">IF(ISNUMBER(R9),D9*R9,0)</f>
+        <v>407250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3358,11 +3381,12 @@
         <v>100.74</v>
       </c>
       <c r="R10" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F10,I10,L10)=0,"Sem cotação",ROUND(P10,2))</f>
+        <v>90.74</v>
       </c>
       <c r="S10" s="12" t="n">
-        <f aca="false">D10*R10</f>
-        <v>381910</v>
+        <f aca="false">IF(ISNUMBER(R10),D10*R10,0)</f>
+        <v>410598.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3422,11 +3446,12 @@
         <v>155</v>
       </c>
       <c r="R11" s="14" t="n">
-        <v>84.4</v>
+        <f aca="false">IF(COUNT(F11,I11,L11)=0,"Sem cotação",ROUND(P11,2))</f>
+        <v>95.31</v>
       </c>
       <c r="S11" s="12" t="n">
-        <f aca="false">D11*R11</f>
-        <v>4582920</v>
+        <f aca="false">IF(ISNUMBER(R11),D11*R11,0)</f>
+        <v>5175333</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3452,7 +3477,7 @@
       <c r="R12" s="15"/>
       <c r="S12" s="7" t="n">
         <f aca="false">SUM(S3:S11)</f>
-        <v>18905067.11</v>
+        <v>20674426.8</v>
       </c>
     </row>
   </sheetData>
@@ -3663,11 +3688,12 @@
         <v>543.33</v>
       </c>
       <c r="R3" s="14" t="n">
-        <v>403.2</v>
+        <f aca="false">IF(COUNT(F3,I3,L3)=0,"Sem cotação",ROUND(P3,2))</f>
+        <v>420</v>
       </c>
       <c r="S3" s="12" t="n">
-        <f aca="false">D3*R3</f>
-        <v>10946880</v>
+        <f aca="false">IF(ISNUMBER(R3),D3*R3,0)</f>
+        <v>11403000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,11 +3753,12 @@
         <v>300</v>
       </c>
       <c r="R4" s="14" t="n">
-        <v>172.8</v>
+        <f aca="false">IF(COUNT(F4,I4,L4)=0,"Sem cotação",ROUND(P4,2))</f>
+        <v>110</v>
       </c>
       <c r="S4" s="12" t="n">
-        <f aca="false">D4*R4</f>
-        <v>703814.4</v>
+        <f aca="false">IF(ISNUMBER(R4),D4*R4,0)</f>
+        <v>448030</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3757,7 +3784,7 @@
       <c r="R5" s="15"/>
       <c r="S5" s="7" t="n">
         <f aca="false">SUM(S3:S4)</f>
-        <v>11650694.4</v>
+        <v>11851030</v>
       </c>
     </row>
   </sheetData>
@@ -3947,11 +3974,12 @@
         <v>90.1</v>
       </c>
       <c r="R3" s="14" t="n">
-        <v>86.28</v>
+        <f aca="false">IF(COUNT(F3,I3,L3)=0,"Sem cotação",ROUND(P3,2))</f>
+        <v>78.4</v>
       </c>
       <c r="S3" s="12" t="n">
-        <f aca="false">D3*R3</f>
-        <v>7775381.04</v>
+        <f aca="false">IF(ISNUMBER(R3),D3*R3,0)</f>
+        <v>7065251.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4011,11 +4039,12 @@
         <v>76.05</v>
       </c>
       <c r="R4" s="14" t="n">
-        <v>69.81</v>
+        <f aca="false">IF(COUNT(F4,I4,L4)=0,"Sem cotação",ROUND(P4,2))</f>
+        <v>53.8</v>
       </c>
       <c r="S4" s="12" t="n">
-        <f aca="false">D4*R4</f>
-        <v>63178.05</v>
+        <f aca="false">IF(ISNUMBER(R4),D4*R4,0)</f>
+        <v>48689</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4075,11 +4104,12 @@
         <v>76.05</v>
       </c>
       <c r="R5" s="14" t="n">
-        <v>69.81</v>
+        <f aca="false">IF(COUNT(F5,I5,L5)=0,"Sem cotação",ROUND(P5,2))</f>
+        <v>53.8</v>
       </c>
       <c r="S5" s="12" t="n">
-        <f aca="false">D5*R5</f>
-        <v>63178.05</v>
+        <f aca="false">IF(ISNUMBER(R5),D5*R5,0)</f>
+        <v>48689</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4139,11 +4169,12 @@
         <v>98.27</v>
       </c>
       <c r="R6" s="14" t="n">
-        <v>90.2</v>
+        <f aca="false">IF(COUNT(F6,I6,L6)=0,"Sem cotação",ROUND(P6,2))</f>
+        <v>83.97</v>
       </c>
       <c r="S6" s="12" t="n">
-        <f aca="false">D6*R6</f>
-        <v>81631</v>
+        <f aca="false">IF(ISNUMBER(R6),D6*R6,0)</f>
+        <v>75992.85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4199,11 +4230,12 @@
         <v>116.21</v>
       </c>
       <c r="R7" s="14" t="n">
-        <v>106.67</v>
+        <f aca="false">IF(COUNT(F7,I7,L7)=0,"Sem cotação",ROUND(P7,2))</f>
+        <v>99.21</v>
       </c>
       <c r="S7" s="12" t="n">
-        <f aca="false">D7*R7</f>
-        <v>146777.92</v>
+        <f aca="false">IF(ISNUMBER(R7),D7*R7,0)</f>
+        <v>136512.96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4263,11 +4295,12 @@
         <v>109.36</v>
       </c>
       <c r="R8" s="14" t="n">
-        <v>104.71</v>
+        <f aca="false">IF(COUNT(F8,I8,L8)=0,"Sem cotação",ROUND(P8,2))</f>
+        <v>80.7</v>
       </c>
       <c r="S8" s="12" t="n">
-        <f aca="false">D8*R8</f>
-        <v>134238.22</v>
+        <f aca="false">IF(ISNUMBER(R8),D8*R8,0)</f>
+        <v>103457.4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4327,11 +4360,12 @@
         <v>90.1</v>
       </c>
       <c r="R9" s="14" t="n">
-        <v>86.28</v>
+        <f aca="false">IF(COUNT(F9,I9,L9)=0,"Sem cotação",ROUND(P9,2))</f>
+        <v>66.5</v>
       </c>
       <c r="S9" s="12" t="n">
-        <f aca="false">D9*R9</f>
-        <v>1285830.84</v>
+        <f aca="false">IF(ISNUMBER(R9),D9*R9,0)</f>
+        <v>991049.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4391,11 +4425,12 @@
         <v>90</v>
       </c>
       <c r="R10" s="14" t="n">
-        <v>90.2</v>
+        <f aca="false">IF(COUNT(F10,I10,L10)=0,"Sem cotação",ROUND(P10,2))</f>
+        <v>82.42</v>
       </c>
       <c r="S10" s="12" t="n">
-        <f aca="false">D10*R10</f>
-        <v>403284.2</v>
+        <f aca="false">IF(ISNUMBER(R10),D10*R10,0)</f>
+        <v>368499.82</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4455,11 +4490,12 @@
         <v>73</v>
       </c>
       <c r="R11" s="14" t="n">
-        <v>69.81</v>
+        <f aca="false">IF(COUNT(F11,I11,L11)=0,"Sem cotação",ROUND(P11,2))</f>
+        <v>72.91</v>
       </c>
       <c r="S11" s="12" t="n">
-        <f aca="false">D11*R11</f>
-        <v>63178.05</v>
+        <f aca="false">IF(ISNUMBER(R11),D11*R11,0)</f>
+        <v>65983.55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4519,11 +4555,12 @@
         <v>96.28</v>
       </c>
       <c r="R12" s="14" t="n">
-        <v>92.16</v>
+        <f aca="false">IF(COUNT(F12,I12,L12)=0,"Sem cotação",ROUND(P12,2))</f>
+        <v>71</v>
       </c>
       <c r="S12" s="12" t="n">
-        <f aca="false">D12*R12</f>
-        <v>83404.8</v>
+        <f aca="false">IF(ISNUMBER(R12),D12*R12,0)</f>
+        <v>64255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4583,11 +4620,12 @@
         <v>167</v>
       </c>
       <c r="R13" s="14" t="n">
-        <v>131.38</v>
+        <f aca="false">IF(COUNT(F13,I13,L13)=0,"Sem cotação",ROUND(P13,2))</f>
+        <v>104.5</v>
       </c>
       <c r="S13" s="12" t="n">
-        <f aca="false">D13*R13</f>
-        <v>118898.9</v>
+        <f aca="false">IF(ISNUMBER(R13),D13*R13,0)</f>
+        <v>94572.5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4647,11 +4685,12 @@
         <v>166</v>
       </c>
       <c r="R14" s="14" t="n">
-        <v>141.17</v>
+        <f aca="false">IF(COUNT(F14,I14,L14)=0,"Sem cotação",ROUND(P14,2))</f>
+        <v>108.75</v>
       </c>
       <c r="S14" s="12" t="n">
-        <f aca="false">D14*R14</f>
-        <v>717567.11</v>
+        <f aca="false">IF(ISNUMBER(R14),D14*R14,0)</f>
+        <v>552776.25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4703,11 +4742,12 @@
         <v>66.5</v>
       </c>
       <c r="R15" s="14" t="n">
-        <v>86.28</v>
+        <f aca="false">IF(COUNT(F15,I15,L15)=0,"Sem cotação",ROUND(P15,2))</f>
+        <v>66.5</v>
       </c>
       <c r="S15" s="12" t="n">
-        <f aca="false">D15*R15</f>
-        <v>78083.4</v>
+        <f aca="false">IF(ISNUMBER(R15),D15*R15,0)</f>
+        <v>60182.5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4759,11 +4799,12 @@
         <v>82.2</v>
       </c>
       <c r="R16" s="14" t="n">
-        <v>106.67</v>
+        <f aca="false">IF(COUNT(F16,I16,L16)=0,"Sem cotação",ROUND(P16,2))</f>
+        <v>82.2</v>
       </c>
       <c r="S16" s="12" t="n">
-        <f aca="false">D16*R16</f>
-        <v>96536.35</v>
+        <f aca="false">IF(ISNUMBER(R16),D16*R16,0)</f>
+        <v>74391</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4815,11 +4856,12 @@
         <v>107.6</v>
       </c>
       <c r="R17" s="14" t="n">
-        <v>139.62</v>
+        <f aca="false">IF(COUNT(F17,I17,L17)=0,"Sem cotação",ROUND(P17,2))</f>
+        <v>107.6</v>
       </c>
       <c r="S17" s="12" t="n">
-        <f aca="false">D17*R17</f>
-        <v>126356.1</v>
+        <f aca="false">IF(ISNUMBER(R17),D17*R17,0)</f>
+        <v>97378</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4871,11 +4913,12 @@
         <v>107.6</v>
       </c>
       <c r="R18" s="14" t="n">
-        <v>139.62</v>
+        <f aca="false">IF(COUNT(F18,I18,L18)=0,"Sem cotação",ROUND(P18,2))</f>
+        <v>107.6</v>
       </c>
       <c r="S18" s="12" t="n">
-        <f aca="false">D18*R18</f>
-        <v>126356.1</v>
+        <f aca="false">IF(ISNUMBER(R18),D18*R18,0)</f>
+        <v>97378</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4927,11 +4970,12 @@
         <v>66.5</v>
       </c>
       <c r="R19" s="14" t="n">
-        <v>86.28</v>
+        <f aca="false">IF(COUNT(F19,I19,L19)=0,"Sem cotação",ROUND(P19,2))</f>
+        <v>66.5</v>
       </c>
       <c r="S19" s="12" t="n">
-        <f aca="false">D19*R19</f>
-        <v>78083.4</v>
+        <f aca="false">IF(ISNUMBER(R19),D19*R19,0)</f>
+        <v>60182.5</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4983,11 +5027,12 @@
         <v>107.6</v>
       </c>
       <c r="R20" s="14" t="n">
-        <v>139.62</v>
+        <f aca="false">IF(COUNT(F20,I20,L20)=0,"Sem cotação",ROUND(P20,2))</f>
+        <v>107.6</v>
       </c>
       <c r="S20" s="12" t="n">
-        <f aca="false">D20*R20</f>
-        <v>126356.1</v>
+        <f aca="false">IF(ISNUMBER(R20),D20*R20,0)</f>
+        <v>97378</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5047,11 +5092,12 @@
         <v>127.89</v>
       </c>
       <c r="R21" s="14" t="n">
-        <v>161.97</v>
+        <f aca="false">IF(COUNT(F21,I21,L21)=0,"Sem cotação",ROUND(P21,2))</f>
+        <v>124.8</v>
       </c>
       <c r="S21" s="12" t="n">
-        <f aca="false">D21*R21</f>
-        <v>500811.24</v>
+        <f aca="false">IF(ISNUMBER(R21),D21*R21,0)</f>
+        <v>385881.6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5111,11 +5157,12 @@
         <v>70.5</v>
       </c>
       <c r="R22" s="14" t="n">
-        <v>88.24</v>
+        <f aca="false">IF(COUNT(F22,I22,L22)=0,"Sem cotação",ROUND(P22,2))</f>
+        <v>68</v>
       </c>
       <c r="S22" s="12" t="n">
-        <f aca="false">D22*R22</f>
-        <v>958286.4</v>
+        <f aca="false">IF(ISNUMBER(R22),D22*R22,0)</f>
+        <v>738480</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5175,11 +5222,12 @@
         <v>104.25</v>
       </c>
       <c r="R23" s="14" t="n">
-        <v>135.3</v>
+        <f aca="false">IF(COUNT(F23,I23,L23)=0,"Sem cotação",ROUND(P23,2))</f>
+        <v>99</v>
       </c>
       <c r="S23" s="12" t="n">
-        <f aca="false">D23*R23</f>
-        <v>24489.3</v>
+        <f aca="false">IF(ISNUMBER(R23),D23*R23,0)</f>
+        <v>17919</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5239,11 +5287,12 @@
         <v>124.8</v>
       </c>
       <c r="R24" s="14" t="n">
-        <v>161.97</v>
+        <f aca="false">IF(COUNT(F24,I24,L24)=0,"Sem cotação",ROUND(P24,2))</f>
+        <v>99</v>
       </c>
       <c r="S24" s="12" t="n">
-        <f aca="false">D24*R24</f>
-        <v>409460.16</v>
+        <f aca="false">IF(ISNUMBER(R24),D24*R24,0)</f>
+        <v>250272</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5303,11 +5352,12 @@
         <v>113</v>
       </c>
       <c r="R25" s="14" t="n">
-        <v>135.3</v>
+        <f aca="false">IF(COUNT(F25,I25,L25)=0,"Sem cotação",ROUND(P25,2))</f>
+        <v>104.25</v>
       </c>
       <c r="S25" s="12" t="n">
-        <f aca="false">D25*R25</f>
-        <v>13124.1</v>
+        <f aca="false">IF(ISNUMBER(R25),D25*R25,0)</f>
+        <v>10112.25</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5367,11 +5417,12 @@
         <v>152</v>
       </c>
       <c r="R26" s="14" t="n">
-        <v>222.37</v>
+        <f aca="false">IF(COUNT(F26,I26,L26)=0,"Sem cotação",ROUND(P26,2))</f>
+        <v>139.6</v>
       </c>
       <c r="S26" s="12" t="n">
-        <f aca="false">D26*R26</f>
-        <v>22681.74</v>
+        <f aca="false">IF(ISNUMBER(R26),D26*R26,0)</f>
+        <v>14239.2</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5431,11 +5482,12 @@
         <v>171.35</v>
       </c>
       <c r="R27" s="14" t="n">
-        <v>222.37</v>
+        <f aca="false">IF(COUNT(F27,I27,L27)=0,"Sem cotação",ROUND(P27,2))</f>
+        <v>166</v>
       </c>
       <c r="S27" s="12" t="n">
-        <f aca="false">D27*R27</f>
-        <v>10673.76</v>
+        <f aca="false">IF(ISNUMBER(R27),D27*R27,0)</f>
+        <v>7968</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5491,11 +5543,12 @@
         <v>235.75</v>
       </c>
       <c r="R28" s="14" t="n">
-        <v>305.91</v>
+        <f aca="false">IF(COUNT(F28,I28,L28)=0,"Sem cotação",ROUND(P28,2))</f>
+        <v>218.13</v>
       </c>
       <c r="S28" s="12" t="n">
-        <f aca="false">D28*R28</f>
-        <v>276848.55</v>
+        <f aca="false">IF(ISNUMBER(R28),D28*R28,0)</f>
+        <v>197407.65</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5547,11 +5600,12 @@
         <v>136</v>
       </c>
       <c r="R29" s="14" t="n">
-        <v>176.48</v>
+        <f aca="false">IF(COUNT(F29,I29,L29)=0,"Sem cotação",ROUND(P29,2))</f>
+        <v>136</v>
       </c>
       <c r="S29" s="12" t="n">
-        <f aca="false">D29*R29</f>
-        <v>8471.04</v>
+        <f aca="false">IF(ISNUMBER(R29),D29*R29,0)</f>
+        <v>6528</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5611,11 +5665,12 @@
         <v>150</v>
       </c>
       <c r="R30" s="14" t="n">
-        <v>143.13</v>
+        <f aca="false">IF(COUNT(F30,I30,L30)=0,"Sem cotação",ROUND(P30,2))</f>
+        <v>149.56</v>
       </c>
       <c r="S30" s="12" t="n">
-        <f aca="false">D30*R30</f>
-        <v>129532.65</v>
+        <f aca="false">IF(ISNUMBER(R30),D30*R30,0)</f>
+        <v>135351.8</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5675,11 +5730,12 @@
         <v>76.05</v>
       </c>
       <c r="R31" s="14" t="n">
-        <v>69.81</v>
+        <f aca="false">IF(COUNT(F31,I31,L31)=0,"Sem cotação",ROUND(P31,2))</f>
+        <v>53.8</v>
       </c>
       <c r="S31" s="12" t="n">
-        <f aca="false">D31*R31</f>
-        <v>63178.05</v>
+        <f aca="false">IF(ISNUMBER(R31),D31*R31,0)</f>
+        <v>48689</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5739,11 +5795,12 @@
         <v>72.91</v>
       </c>
       <c r="R32" s="14" t="n">
-        <v>69.81</v>
+        <f aca="false">IF(COUNT(F32,I32,L32)=0,"Sem cotação",ROUND(P32,2))</f>
+        <v>53.8</v>
       </c>
       <c r="S32" s="12" t="n">
-        <f aca="false">D32*R32</f>
-        <v>63178.05</v>
+        <f aca="false">IF(ISNUMBER(R32),D32*R32,0)</f>
+        <v>48689</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5803,11 +5860,12 @@
         <v>64.31</v>
       </c>
       <c r="R33" s="14" t="n">
-        <v>61.57</v>
+        <f aca="false">IF(COUNT(F33,I33,L33)=0,"Sem cotação",ROUND(P33,2))</f>
+        <v>43.9</v>
       </c>
       <c r="S33" s="12" t="n">
-        <f aca="false">D33*R33</f>
-        <v>1350968.94</v>
+        <f aca="false">IF(ISNUMBER(R33),D33*R33,0)</f>
+        <v>963253.8</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5867,11 +5925,12 @@
         <v>94.22</v>
       </c>
       <c r="R34" s="14" t="n">
-        <v>90.2</v>
+        <f aca="false">IF(COUNT(F34,I34,L34)=0,"Sem cotação",ROUND(P34,2))</f>
+        <v>69.5</v>
       </c>
       <c r="S34" s="12" t="n">
-        <f aca="false">D34*R34</f>
-        <v>81631</v>
+        <f aca="false">IF(ISNUMBER(R34),D34*R34,0)</f>
+        <v>62897.5</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5931,11 +5990,12 @@
         <v>137.21</v>
       </c>
       <c r="R35" s="14" t="n">
-        <v>131.38</v>
+        <f aca="false">IF(COUNT(F35,I35,L35)=0,"Sem cotação",ROUND(P35,2))</f>
+        <v>101.25</v>
       </c>
       <c r="S35" s="12" t="n">
-        <f aca="false">D35*R35</f>
-        <v>118898.9</v>
+        <f aca="false">IF(ISNUMBER(R35),D35*R35,0)</f>
+        <v>91631.25</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5995,11 +6055,12 @@
         <v>641.01</v>
       </c>
       <c r="R36" s="14" t="n">
-        <v>613.78</v>
+        <f aca="false">IF(COUNT(F36,I36,L36)=0,"Sem cotação",ROUND(P36,2))</f>
+        <v>600</v>
       </c>
       <c r="S36" s="12" t="n">
-        <f aca="false">D36*R36</f>
-        <v>555470.9</v>
+        <f aca="false">IF(ISNUMBER(R36),D36*R36,0)</f>
+        <v>543000</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6059,11 +6120,12 @@
         <v>638</v>
       </c>
       <c r="R37" s="14" t="n">
-        <v>278.43</v>
+        <f aca="false">IF(COUNT(F37,I37,L37)=0,"Sem cotação",ROUND(P37,2))</f>
+        <v>290.89</v>
       </c>
       <c r="S37" s="12" t="n">
-        <f aca="false">D37*R37</f>
-        <v>67380.06</v>
+        <f aca="false">IF(ISNUMBER(R37),D37*R37,0)</f>
+        <v>70395.38</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6123,11 +6185,12 @@
         <v>653.36</v>
       </c>
       <c r="R38" s="14" t="n">
-        <v>521.28</v>
+        <f aca="false">IF(COUNT(F38,I38,L38)=0,"Sem cotação",ROUND(P38,2))</f>
+        <v>482</v>
       </c>
       <c r="S38" s="12" t="n">
-        <f aca="false">D38*R38</f>
-        <v>471758.4</v>
+        <f aca="false">IF(ISNUMBER(R38),D38*R38,0)</f>
+        <v>436210</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6187,11 +6250,12 @@
         <v>18.32</v>
       </c>
       <c r="R39" s="14" t="n">
-        <v>15.13</v>
+        <f aca="false">IF(COUNT(F39,I39,L39)=0,"Sem cotação",ROUND(P39,2))</f>
+        <v>15.82</v>
       </c>
       <c r="S39" s="12" t="n">
-        <f aca="false">D39*R39</f>
-        <v>13692.65</v>
+        <f aca="false">IF(ISNUMBER(R39),D39*R39,0)</f>
+        <v>14317.1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6251,11 +6315,12 @@
         <v>257.8</v>
       </c>
       <c r="R40" s="14" t="n">
-        <v>334.54</v>
+        <f aca="false">IF(COUNT(F40,I40,L40)=0,"Sem cotação",ROUND(P40,2))</f>
+        <v>180</v>
       </c>
       <c r="S40" s="12" t="n">
-        <f aca="false">D40*R40</f>
-        <v>276330.04</v>
+        <f aca="false">IF(ISNUMBER(R40),D40*R40,0)</f>
+        <v>148680</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6315,11 +6380,12 @@
         <v>238</v>
       </c>
       <c r="R41" s="14" t="n">
-        <v>178.44</v>
+        <f aca="false">IF(COUNT(F41,I41,L41)=0,"Sem cotação",ROUND(P41,2))</f>
+        <v>186.38</v>
       </c>
       <c r="S41" s="12" t="n">
-        <f aca="false">D41*R41</f>
-        <v>161488.2</v>
+        <f aca="false">IF(ISNUMBER(R41),D41*R41,0)</f>
+        <v>168673.9</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6375,11 +6441,12 @@
         <v>68</v>
       </c>
       <c r="R42" s="14" t="n">
-        <v>88.24</v>
+        <f aca="false">IF(COUNT(F42,I42,L42)=0,"Sem cotação",ROUND(P42,2))</f>
+        <v>49</v>
       </c>
       <c r="S42" s="12" t="n">
-        <f aca="false">D42*R42</f>
-        <v>79857.2</v>
+        <f aca="false">IF(ISNUMBER(R42),D42*R42,0)</f>
+        <v>44345</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6439,11 +6506,12 @@
         <v>78.5</v>
       </c>
       <c r="R43" s="14" t="n">
-        <v>53.33</v>
+        <f aca="false">IF(COUNT(F43,I43,L43)=0,"Sem cotação",ROUND(P43,2))</f>
+        <v>41.1</v>
       </c>
       <c r="S43" s="12" t="n">
-        <f aca="false">D43*R43</f>
-        <v>79781.68</v>
+        <f aca="false">IF(ISNUMBER(R43),D43*R43,0)</f>
+        <v>61485.6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6503,11 +6571,12 @@
         <v>90</v>
       </c>
       <c r="R44" s="14" t="n">
-        <v>90.2</v>
+        <f aca="false">IF(COUNT(F44,I44,L44)=0,"Sem cotação",ROUND(P44,2))</f>
+        <v>78.5</v>
       </c>
       <c r="S44" s="12" t="n">
-        <f aca="false">D44*R44</f>
-        <v>134939.2</v>
+        <f aca="false">IF(ISNUMBER(R44),D44*R44,0)</f>
+        <v>117436</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6567,11 +6636,12 @@
         <v>115.53</v>
       </c>
       <c r="R45" s="14" t="n">
-        <v>110.59</v>
+        <f aca="false">IF(COUNT(F45,I45,L45)=0,"Sem cotação",ROUND(P45,2))</f>
+        <v>107</v>
       </c>
       <c r="S45" s="12" t="n">
-        <f aca="false">D45*R45</f>
-        <v>70777.6</v>
+        <f aca="false">IF(ISNUMBER(R45),D45*R45,0)</f>
+        <v>68480</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6631,11 +6701,12 @@
         <v>121</v>
       </c>
       <c r="R46" s="14" t="n">
-        <v>110.59</v>
+        <f aca="false">IF(COUNT(F46,I46,L46)=0,"Sem cotação",ROUND(P46,2))</f>
+        <v>115.53</v>
       </c>
       <c r="S46" s="12" t="n">
-        <f aca="false">D46*R46</f>
-        <v>555935.93</v>
+        <f aca="false">IF(ISNUMBER(R46),D46*R46,0)</f>
+        <v>580769.31</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6695,11 +6766,12 @@
         <v>137.21</v>
       </c>
       <c r="R47" s="14" t="n">
-        <v>131.38</v>
+        <f aca="false">IF(COUNT(F47,I47,L47)=0,"Sem cotação",ROUND(P47,2))</f>
+        <v>101.25</v>
       </c>
       <c r="S47" s="12" t="n">
-        <f aca="false">D47*R47</f>
-        <v>417000.12</v>
+        <f aca="false">IF(ISNUMBER(R47),D47*R47,0)</f>
+        <v>321367.5</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6759,11 +6831,12 @@
         <v>180.2</v>
       </c>
       <c r="R48" s="14" t="n">
-        <v>172.56</v>
+        <f aca="false">IF(COUNT(F48,I48,L48)=0,"Sem cotação",ROUND(P48,2))</f>
+        <v>133</v>
       </c>
       <c r="S48" s="12" t="n">
-        <f aca="false">D48*R48</f>
-        <v>547705.44</v>
+        <f aca="false">IF(ISNUMBER(R48),D48*R48,0)</f>
+        <v>422142</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6823,11 +6896,12 @@
         <v>223.2</v>
       </c>
       <c r="R49" s="14" t="n">
-        <v>213.75</v>
+        <f aca="false">IF(COUNT(F49,I49,L49)=0,"Sem cotação",ROUND(P49,2))</f>
+        <v>164.75</v>
       </c>
       <c r="S49" s="12" t="n">
-        <f aca="false">D49*R49</f>
-        <v>580331.25</v>
+        <f aca="false">IF(ISNUMBER(R49),D49*R49,0)</f>
+        <v>447296.25</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6887,11 +6961,12 @@
         <v>248.99</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>238.46</v>
+        <f aca="false">IF(COUNT(F50,I50,L50)=0,"Sem cotação",ROUND(P50,2))</f>
+        <v>183.8</v>
       </c>
       <c r="S50" s="12" t="n">
-        <f aca="false">D50*R50</f>
-        <v>1198738.42</v>
+        <f aca="false">IF(ISNUMBER(R50),D50*R50,0)</f>
+        <v>923962.6</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6951,11 +7026,12 @@
         <v>223.2</v>
       </c>
       <c r="R51" s="14" t="n">
-        <v>213.75</v>
+        <f aca="false">IF(COUNT(F51,I51,L51)=0,"Sem cotação",ROUND(P51,2))</f>
+        <v>164.75</v>
       </c>
       <c r="S51" s="12" t="n">
-        <f aca="false">D51*R51</f>
-        <v>1074521.25</v>
+        <f aca="false">IF(ISNUMBER(R51),D51*R51,0)</f>
+        <v>828198.25</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7015,11 +7091,12 @@
         <v>248.99</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>238.46</v>
+        <f aca="false">IF(COUNT(F52,I52,L52)=0,"Sem cotação",ROUND(P52,2))</f>
+        <v>183.8</v>
       </c>
       <c r="S52" s="12" t="n">
-        <f aca="false">D52*R52</f>
-        <v>1309383.86</v>
+        <f aca="false">IF(ISNUMBER(R52),D52*R52,0)</f>
+        <v>1009245.8</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7079,11 +7156,12 @@
         <v>137.21</v>
       </c>
       <c r="R53" s="14" t="n">
-        <v>131.38</v>
+        <f aca="false">IF(COUNT(F53,I53,L53)=0,"Sem cotação",ROUND(P53,2))</f>
+        <v>101.25</v>
       </c>
       <c r="S53" s="12" t="n">
-        <f aca="false">D53*R53</f>
-        <v>118898.9</v>
+        <f aca="false">IF(ISNUMBER(R53),D53*R53,0)</f>
+        <v>91631.25</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7143,11 +7221,12 @@
         <v>71.36</v>
       </c>
       <c r="R54" s="14" t="n">
-        <v>65.49</v>
+        <f aca="false">IF(COUNT(F54,I54,L54)=0,"Sem cotação",ROUND(P54,2))</f>
+        <v>56.5</v>
       </c>
       <c r="S54" s="12" t="n">
-        <f aca="false">D54*R54</f>
-        <v>59268.45</v>
+        <f aca="false">IF(ISNUMBER(R54),D54*R54,0)</f>
+        <v>51132.5</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7207,11 +7286,12 @@
         <v>343.95</v>
       </c>
       <c r="R55" s="14" t="n">
-        <v>315.7</v>
+        <f aca="false">IF(COUNT(F55,I55,L55)=0,"Sem cotação",ROUND(P55,2))</f>
+        <v>329.77</v>
       </c>
       <c r="S55" s="12" t="n">
-        <f aca="false">D55*R55</f>
-        <v>285708.5</v>
+        <f aca="false">IF(ISNUMBER(R55),D55*R55,0)</f>
+        <v>298441.85</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7271,11 +7351,12 @@
         <v>252.11</v>
       </c>
       <c r="R56" s="14" t="n">
-        <v>233.33</v>
+        <f aca="false">IF(COUNT(F56,I56,L56)=0,"Sem cotação",ROUND(P56,2))</f>
+        <v>243.78</v>
       </c>
       <c r="S56" s="12" t="n">
-        <f aca="false">D56*R56</f>
-        <v>211163.65</v>
+        <f aca="false">IF(ISNUMBER(R56),D56*R56,0)</f>
+        <v>220620.9</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7331,11 +7412,12 @@
         <v>86.7</v>
       </c>
       <c r="R57" s="14" t="n">
-        <v>112.55</v>
+        <f aca="false">IF(COUNT(F57,I57,L57)=0,"Sem cotação",ROUND(P57,2))</f>
+        <v>53.35</v>
       </c>
       <c r="S57" s="12" t="n">
-        <f aca="false">D57*R57</f>
-        <v>101857.75</v>
+        <f aca="false">IF(ISNUMBER(R57),D57*R57,0)</f>
+        <v>48281.75</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7382,12 +7464,13 @@
         <f aca="false">IF(COUNT(F58,I58,L58)=0,"",MAX(F58,I58,L58))</f>
         <v/>
       </c>
-      <c r="R58" s="14" t="n">
-        <v>145.49</v>
+      <c r="R58" s="14" t="str">
+        <f aca="false">IF(COUNT(F58,I58,L58)=0,"Sem cotação",ROUND(P58,2))</f>
+        <v>Sem cotação</v>
       </c>
       <c r="S58" s="12" t="n">
-        <f aca="false">D58*R58</f>
-        <v>131668.45</v>
+        <f aca="false">IF(ISNUMBER(R58),D58*R58,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7447,11 +7530,12 @@
         <v>610.5</v>
       </c>
       <c r="R59" s="14" t="n">
-        <v>398.07</v>
+        <f aca="false">IF(COUNT(F59,I59,L59)=0,"Sem cotação",ROUND(P59,2))</f>
+        <v>415.75</v>
       </c>
       <c r="S59" s="12" t="n">
-        <f aca="false">D59*R59</f>
-        <v>78021.72</v>
+        <f aca="false">IF(ISNUMBER(R59),D59*R59,0)</f>
+        <v>81487</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7511,11 +7595,12 @@
         <v>123.5</v>
       </c>
       <c r="R60" s="14" t="n">
-        <v>93.33</v>
+        <f aca="false">IF(COUNT(F60,I60,L60)=0,"Sem cotação",ROUND(P60,2))</f>
+        <v>71.9</v>
       </c>
       <c r="S60" s="12" t="n">
-        <f aca="false">D60*R60</f>
-        <v>84463.65</v>
+        <f aca="false">IF(ISNUMBER(R60),D60*R60,0)</f>
+        <v>65069.5</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7567,11 +7652,12 @@
         <v>53.8</v>
       </c>
       <c r="R61" s="14" t="n">
-        <v>69.81</v>
+        <f aca="false">IF(COUNT(F61,I61,L61)=0,"Sem cotação",ROUND(P61,2))</f>
+        <v>53.8</v>
       </c>
       <c r="S61" s="12" t="n">
-        <f aca="false">D61*R61</f>
-        <v>63178.05</v>
+        <f aca="false">IF(ISNUMBER(R61),D61*R61,0)</f>
+        <v>48689</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7631,11 +7717,12 @@
         <v>339.58</v>
       </c>
       <c r="R62" s="14" t="n">
-        <v>317.66</v>
+        <f aca="false">IF(COUNT(F62,I62,L62)=0,"Sem cotação",ROUND(P62,2))</f>
+        <v>331.82</v>
       </c>
       <c r="S62" s="12" t="n">
-        <f aca="false">D62*R62</f>
-        <v>287482.3</v>
+        <f aca="false">IF(ISNUMBER(R62),D62*R62,0)</f>
+        <v>300297.1</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7691,11 +7778,12 @@
         <v>143.39</v>
       </c>
       <c r="R63" s="14" t="n">
-        <v>137.26</v>
+        <f aca="false">IF(COUNT(F63,I63,L63)=0,"Sem cotação",ROUND(P63,2))</f>
+        <v>124.57</v>
       </c>
       <c r="S63" s="12" t="n">
-        <f aca="false">D63*R63</f>
-        <v>16471.2</v>
+        <f aca="false">IF(ISNUMBER(R63),D63*R63,0)</f>
+        <v>14948.4</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7755,11 +7843,12 @@
         <v>259.88</v>
       </c>
       <c r="R64" s="14" t="n">
-        <v>231.37</v>
+        <f aca="false">IF(COUNT(F64,I64,L64)=0,"Sem cotação",ROUND(P64,2))</f>
+        <v>240.59</v>
       </c>
       <c r="S64" s="12" t="n">
-        <f aca="false">D64*R64</f>
-        <v>31234.95</v>
+        <f aca="false">IF(ISNUMBER(R64),D64*R64,0)</f>
+        <v>32479.65</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7819,11 +7908,12 @@
         <v>514.65</v>
       </c>
       <c r="R65" s="14" t="n">
-        <v>398.07</v>
+        <f aca="false">IF(COUNT(F65,I65,L65)=0,"Sem cotação",ROUND(P65,2))</f>
+        <v>415.75</v>
       </c>
       <c r="S65" s="12" t="n">
-        <f aca="false">D65*R65</f>
-        <v>28661.04</v>
+        <f aca="false">IF(ISNUMBER(R65),D65*R65,0)</f>
+        <v>29934</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7879,11 +7969,12 @@
         <v>156</v>
       </c>
       <c r="R66" s="14" t="n">
-        <v>94.11</v>
+        <f aca="false">IF(COUNT(F66,I66,L66)=0,"Sem cotação",ROUND(P66,2))</f>
+        <v>114.25</v>
       </c>
       <c r="S66" s="12" t="n">
-        <f aca="false">D66*R66</f>
-        <v>6775.92</v>
+        <f aca="false">IF(ISNUMBER(R66),D66*R66,0)</f>
+        <v>8226</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7909,7 +8000,7 @@
       <c r="R67" s="15"/>
       <c r="S67" s="7" t="n">
         <f aca="false">SUM(S3:S66)</f>
-        <v>24700500.24</v>
+        <v>20579182.67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>